<commit_message>
Add data for 2026-09-18
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-ytd.xlsx
+++ b/output/cta-violent-crime-ytd.xlsx
@@ -28,80 +28,80 @@
     <sheet name="Belmont Cragin" sheetId="19" r:id="rId19"/>
     <sheet name="West Loop" sheetId="20" r:id="rId20"/>
     <sheet name="Uptown" sheetId="21" r:id="rId21"/>
-    <sheet name="Lake View" sheetId="22" r:id="rId22"/>
-    <sheet name="Grand Boulevard" sheetId="23" r:id="rId23"/>
-    <sheet name="West Town" sheetId="24" r:id="rId24"/>
-    <sheet name="Englewood" sheetId="25" r:id="rId25"/>
-    <sheet name="Greektown" sheetId="26" r:id="rId26"/>
-    <sheet name="Edgewater" sheetId="27" r:id="rId27"/>
-    <sheet name="Little Italy, UIC" sheetId="28" r:id="rId28"/>
-    <sheet name="Gage Park" sheetId="29" r:id="rId29"/>
-    <sheet name="Humboldt Park" sheetId="30" r:id="rId30"/>
-    <sheet name="Lower West Side" sheetId="31" r:id="rId31"/>
-    <sheet name="Sheffield &amp; DePaul" sheetId="32" r:id="rId32"/>
-    <sheet name="Norwood Park" sheetId="33" r:id="rId33"/>
-    <sheet name="Garfield Park" sheetId="34" r:id="rId34"/>
-    <sheet name="Wrigleyville" sheetId="35" r:id="rId35"/>
-    <sheet name="Auburn Gresham" sheetId="36" r:id="rId36"/>
-    <sheet name="Rogers Park" sheetId="37" r:id="rId37"/>
-    <sheet name="Washington Park" sheetId="38" r:id="rId38"/>
-    <sheet name="Chicago Lawn" sheetId="39" r:id="rId39"/>
-    <sheet name="Kenwood" sheetId="40" r:id="rId40"/>
-    <sheet name="Calumet Heights" sheetId="41" r:id="rId41"/>
-    <sheet name="Hyde Park" sheetId="42" r:id="rId42"/>
-    <sheet name="Fuller Park" sheetId="43" r:id="rId43"/>
-    <sheet name="South Chicago" sheetId="44" r:id="rId44"/>
-    <sheet name="Armour Square" sheetId="45" r:id="rId45"/>
-    <sheet name="Douglas" sheetId="46" r:id="rId46"/>
-    <sheet name="United Center" sheetId="47" r:id="rId47"/>
-    <sheet name="Grant Park" sheetId="48" r:id="rId48"/>
-    <sheet name="Jefferson Park" sheetId="49" r:id="rId49"/>
-    <sheet name="Streeterville" sheetId="50" r:id="rId50"/>
-    <sheet name="Millenium Park" sheetId="51" r:id="rId51"/>
-    <sheet name="River North" sheetId="52" r:id="rId52"/>
-    <sheet name="Beverly" sheetId="53" r:id="rId53"/>
-    <sheet name="South Deering" sheetId="54" r:id="rId54"/>
-    <sheet name="West Elsdon" sheetId="55" r:id="rId55"/>
-    <sheet name="Pullman" sheetId="56" r:id="rId56"/>
-    <sheet name="West Pullman" sheetId="57" r:id="rId57"/>
-    <sheet name="Morgan Park" sheetId="58" r:id="rId58"/>
-    <sheet name="Wicker Park" sheetId="59" r:id="rId59"/>
-    <sheet name="Little Village" sheetId="60" r:id="rId60"/>
-    <sheet name="Irving Park" sheetId="61" r:id="rId61"/>
-    <sheet name="Jackson Park" sheetId="62" r:id="rId62"/>
-    <sheet name="Brighton Park" sheetId="63" r:id="rId63"/>
-    <sheet name="Bridgeport" sheetId="64" r:id="rId64"/>
-    <sheet name="Clearing" sheetId="65" r:id="rId65"/>
-    <sheet name="Mckinley Park" sheetId="66" r:id="rId66"/>
-    <sheet name="Chinatown" sheetId="67" r:id="rId67"/>
-    <sheet name="Bucktown" sheetId="68" r:id="rId68"/>
-    <sheet name="Ukrainian Village" sheetId="69" r:id="rId69"/>
-    <sheet name="Ashburn" sheetId="70" r:id="rId70"/>
-    <sheet name="Washington Heights" sheetId="71" r:id="rId71"/>
-    <sheet name="Printers Row" sheetId="72" r:id="rId72"/>
-    <sheet name="Logan Square" sheetId="73" r:id="rId73"/>
-    <sheet name="Lincoln Park" sheetId="74" r:id="rId74"/>
-    <sheet name="Lincoln Square" sheetId="75" r:id="rId75"/>
-    <sheet name="Archer Heights" sheetId="76" r:id="rId76"/>
-    <sheet name="Avalon Park" sheetId="77" r:id="rId77"/>
-    <sheet name="Burnside" sheetId="78" r:id="rId78"/>
-    <sheet name="East Side" sheetId="79" r:id="rId79"/>
-    <sheet name="Portage Park" sheetId="80" r:id="rId80"/>
-    <sheet name="Montclare" sheetId="81" r:id="rId81"/>
-    <sheet name="Hermosa" sheetId="82" r:id="rId82"/>
-    <sheet name="West Ridge" sheetId="83" r:id="rId83"/>
-    <sheet name="North Park" sheetId="84" r:id="rId84"/>
-    <sheet name="North Center" sheetId="85" r:id="rId85"/>
-    <sheet name="Magnificent Mile" sheetId="86" r:id="rId86"/>
-    <sheet name="Riverdale" sheetId="87" r:id="rId87"/>
-    <sheet name="Galewood" sheetId="88" r:id="rId88"/>
-    <sheet name="Gold Coast" sheetId="89" r:id="rId89"/>
-    <sheet name="Mount Greenwood" sheetId="90" r:id="rId90"/>
-    <sheet name="West Lawn" sheetId="91" r:id="rId91"/>
-    <sheet name="Boystown" sheetId="92" r:id="rId92"/>
-    <sheet name="East Village" sheetId="93" r:id="rId93"/>
-    <sheet name="Dunning" sheetId="94" r:id="rId94"/>
-    <sheet name="Hegewisch" sheetId="95" r:id="rId95"/>
+    <sheet name="Hegewisch" sheetId="22" r:id="rId22"/>
+    <sheet name="Lake View" sheetId="23" r:id="rId23"/>
+    <sheet name="Grand Boulevard" sheetId="24" r:id="rId24"/>
+    <sheet name="West Town" sheetId="25" r:id="rId25"/>
+    <sheet name="Englewood" sheetId="26" r:id="rId26"/>
+    <sheet name="Greektown" sheetId="27" r:id="rId27"/>
+    <sheet name="Edgewater" sheetId="28" r:id="rId28"/>
+    <sheet name="Little Italy, UIC" sheetId="29" r:id="rId29"/>
+    <sheet name="Gage Park" sheetId="30" r:id="rId30"/>
+    <sheet name="Humboldt Park" sheetId="31" r:id="rId31"/>
+    <sheet name="Lower West Side" sheetId="32" r:id="rId32"/>
+    <sheet name="Sheffield &amp; DePaul" sheetId="33" r:id="rId33"/>
+    <sheet name="Norwood Park" sheetId="34" r:id="rId34"/>
+    <sheet name="Garfield Park" sheetId="35" r:id="rId35"/>
+    <sheet name="Wrigleyville" sheetId="36" r:id="rId36"/>
+    <sheet name="Auburn Gresham" sheetId="37" r:id="rId37"/>
+    <sheet name="Rogers Park" sheetId="38" r:id="rId38"/>
+    <sheet name="Washington Park" sheetId="39" r:id="rId39"/>
+    <sheet name="Chicago Lawn" sheetId="40" r:id="rId40"/>
+    <sheet name="Kenwood" sheetId="41" r:id="rId41"/>
+    <sheet name="Calumet Heights" sheetId="42" r:id="rId42"/>
+    <sheet name="Hyde Park" sheetId="43" r:id="rId43"/>
+    <sheet name="Fuller Park" sheetId="44" r:id="rId44"/>
+    <sheet name="South Chicago" sheetId="45" r:id="rId45"/>
+    <sheet name="Armour Square" sheetId="46" r:id="rId46"/>
+    <sheet name="Douglas" sheetId="47" r:id="rId47"/>
+    <sheet name="United Center" sheetId="48" r:id="rId48"/>
+    <sheet name="Grant Park" sheetId="49" r:id="rId49"/>
+    <sheet name="Jefferson Park" sheetId="50" r:id="rId50"/>
+    <sheet name="Streeterville" sheetId="51" r:id="rId51"/>
+    <sheet name="Millenium Park" sheetId="52" r:id="rId52"/>
+    <sheet name="River North" sheetId="53" r:id="rId53"/>
+    <sheet name="Beverly" sheetId="54" r:id="rId54"/>
+    <sheet name="South Deering" sheetId="55" r:id="rId55"/>
+    <sheet name="West Elsdon" sheetId="56" r:id="rId56"/>
+    <sheet name="Pullman" sheetId="57" r:id="rId57"/>
+    <sheet name="West Pullman" sheetId="58" r:id="rId58"/>
+    <sheet name="Morgan Park" sheetId="59" r:id="rId59"/>
+    <sheet name="Wicker Park" sheetId="60" r:id="rId60"/>
+    <sheet name="Little Village" sheetId="61" r:id="rId61"/>
+    <sheet name="Irving Park" sheetId="62" r:id="rId62"/>
+    <sheet name="Jackson Park" sheetId="63" r:id="rId63"/>
+    <sheet name="Brighton Park" sheetId="64" r:id="rId64"/>
+    <sheet name="Bridgeport" sheetId="65" r:id="rId65"/>
+    <sheet name="Clearing" sheetId="66" r:id="rId66"/>
+    <sheet name="Mckinley Park" sheetId="67" r:id="rId67"/>
+    <sheet name="Chinatown" sheetId="68" r:id="rId68"/>
+    <sheet name="Bucktown" sheetId="69" r:id="rId69"/>
+    <sheet name="Ukrainian Village" sheetId="70" r:id="rId70"/>
+    <sheet name="Ashburn" sheetId="71" r:id="rId71"/>
+    <sheet name="Washington Heights" sheetId="72" r:id="rId72"/>
+    <sheet name="Printers Row" sheetId="73" r:id="rId73"/>
+    <sheet name="Logan Square" sheetId="74" r:id="rId74"/>
+    <sheet name="Lincoln Park" sheetId="75" r:id="rId75"/>
+    <sheet name="Lincoln Square" sheetId="76" r:id="rId76"/>
+    <sheet name="Archer Heights" sheetId="77" r:id="rId77"/>
+    <sheet name="Avalon Park" sheetId="78" r:id="rId78"/>
+    <sheet name="Burnside" sheetId="79" r:id="rId79"/>
+    <sheet name="East Side" sheetId="80" r:id="rId80"/>
+    <sheet name="Portage Park" sheetId="81" r:id="rId81"/>
+    <sheet name="Montclare" sheetId="82" r:id="rId82"/>
+    <sheet name="Hermosa" sheetId="83" r:id="rId83"/>
+    <sheet name="West Ridge" sheetId="84" r:id="rId84"/>
+    <sheet name="North Park" sheetId="85" r:id="rId85"/>
+    <sheet name="North Center" sheetId="86" r:id="rId86"/>
+    <sheet name="Magnificent Mile" sheetId="87" r:id="rId87"/>
+    <sheet name="Riverdale" sheetId="88" r:id="rId88"/>
+    <sheet name="Galewood" sheetId="89" r:id="rId89"/>
+    <sheet name="Gold Coast" sheetId="90" r:id="rId90"/>
+    <sheet name="Mount Greenwood" sheetId="91" r:id="rId91"/>
+    <sheet name="West Lawn" sheetId="92" r:id="rId92"/>
+    <sheet name="Boystown" sheetId="93" r:id="rId93"/>
+    <sheet name="East Village" sheetId="94" r:id="rId94"/>
+    <sheet name="Dunning" sheetId="95" r:id="rId95"/>
     <sheet name="Andersonville" sheetId="96" r:id="rId96"/>
     <sheet name="Garfield Ridge" sheetId="97" r:id="rId97"/>
   </sheets>
@@ -110,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="104">
   <si>
     <t>crime_category</t>
   </si>
@@ -930,7 +930,7 @@
         <v>181</v>
       </c>
       <c r="M3">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>657</v>
       </c>
       <c r="M7">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -4222,6 +4222,9 @@
       <c r="G39">
         <v>1</v>
       </c>
+      <c r="M39">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" spans="1:13">
       <c r="A40" s="2" t="s">
@@ -6204,7 +6207,7 @@
         <v>657</v>
       </c>
       <c r="M98">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -6773,6 +6776,84 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -7018,7 +7099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7226,7 +7307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7440,7 +7521,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7695,7 +7776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7830,220 +7911,6 @@
       </c>
       <c r="J6">
         <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-      <c r="H5">
-        <v>11</v>
-      </c>
-      <c r="I5">
-        <v>6</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>8</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>11</v>
-      </c>
-      <c r="I6">
-        <v>10</v>
-      </c>
-      <c r="J6">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <v>7</v>
-      </c>
-      <c r="L6">
-        <v>7</v>
-      </c>
-      <c r="M6">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -8117,12 +7984,15 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="G2">
         <v>1</v>
       </c>
       <c r="I2">
@@ -8132,66 +8002,45 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
       <c r="M4">
         <v>1</v>
       </c>
@@ -8201,40 +8050,40 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F5">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -8242,40 +8091,40 @@
         <v>6</v>
       </c>
       <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
         <v>8</v>
       </c>
-      <c r="C6">
+      <c r="G6">
+        <v>8</v>
+      </c>
+      <c r="H6">
+        <v>11</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
+      </c>
+      <c r="J6">
+        <v>9</v>
+      </c>
+      <c r="K6">
         <v>7</v>
       </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>14</v>
-      </c>
-      <c r="F6">
-        <v>23</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>12</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>10</v>
-      </c>
-      <c r="K6">
-        <v>25</v>
-      </c>
       <c r="L6">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="M6">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -8285,7 +8134,7 @@
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -8300,9 +8149,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8325,152 +8175,188 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>12</v>
+      </c>
+      <c r="F5">
+        <v>21</v>
+      </c>
+      <c r="G5">
+        <v>13</v>
+      </c>
+      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5">
         <v>7</v>
       </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
       <c r="J5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="L5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J6">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>19</v>
+      </c>
+      <c r="M6">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -8733,6 +8619,201 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>6</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -8951,7 +9032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9142,7 +9223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9356,7 +9437,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9528,7 +9609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9776,196 +9857,6 @@
       </c>
       <c r="M7">
         <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -10039,59 +9930,44 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
       <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="M3">
         <v>2</v>
       </c>
     </row>
@@ -10099,7 +9975,7 @@
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
@@ -10107,41 +9983,29 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>13</v>
-      </c>
       <c r="C5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -10149,40 +10013,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -10255,35 +10119,32 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>2</v>
+      <c r="H2">
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -10291,36 +10152,27 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3">
-        <v>6</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
         <v>2</v>
       </c>
     </row>
@@ -10328,20 +10180,8 @@
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
+      <c r="C4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -10349,40 +10189,40 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G5">
         <v>6</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -10390,40 +10230,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -10497,19 +10337,31 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
         <v>2</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
       <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
         <v>2</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -10520,19 +10372,22 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3">
         <v>2</v>
@@ -10541,21 +10396,33 @@
         <v>2</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
       <c r="L4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -10563,40 +10430,40 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>7</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -10604,40 +10471,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="I6">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>13</v>
+      </c>
+      <c r="K6">
+        <v>19</v>
+      </c>
+      <c r="L6">
+        <v>17</v>
+      </c>
+      <c r="M6">
         <v>9</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>4</v>
-      </c>
-      <c r="I6">
-        <v>10</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -10710,68 +10577,65 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="J2">
         <v>2</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
         <v>2</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -10780,22 +10644,28 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>8</v>
       </c>
       <c r="J5">
         <v>2</v>
@@ -10805,6 +10675,9 @@
       </c>
       <c r="L5">
         <v>1</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -10812,40 +10685,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
         <v>8</v>
       </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
       <c r="H6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6">
         <v>2</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -11113,6 +10986,214 @@
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -11227,7 +11308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -11390,7 +11471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -11555,7 +11636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -11772,7 +11853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -11978,7 +12059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12201,7 +12282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12402,7 +12483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12625,7 +12706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12689,208 +12770,6 @@
       </c>
       <c r="D5">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>3</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>7</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6">
-        <v>8</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -13085,6 +12964,208 @@
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>7</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>8</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -13192,7 +13273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13240,7 +13321,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13463,7 +13544,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13516,7 +13597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13670,7 +13751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13813,7 +13894,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13901,7 +13982,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14077,7 +14158,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14201,167 +14282,6 @@
       </c>
       <c r="J5">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -14606,25 +14526,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C1" s="1">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="D1" s="1">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="E1" s="1">
         <v>2019</v>
       </c>
       <c r="F1" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="G1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="H1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="I1" s="1">
         <v>2024</v>
@@ -14640,13 +14560,10 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="H2">
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="K2">
         <v>1</v>
       </c>
     </row>
@@ -14654,13 +14571,16 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
         <v>1</v>
       </c>
       <c r="K3">
@@ -14680,27 +14600,27 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="K5">
         <v>1</v>
       </c>
     </row>
@@ -14709,31 +14629,31 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6">
         <v>2</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6">
         <v>4</v>
@@ -14745,6 +14665,167 @@
 </file>
 
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14955,7 +15036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15082,7 +15163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15236,7 +15317,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15407,7 +15488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15545,7 +15626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15695,7 +15776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15917,7 +15998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16020,82 +16101,6 @@
         <v>2</v>
       </c>
       <c r="H5">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -16341,6 +16346,82 @@
 
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -16494,7 +16575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16660,7 +16741,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16831,223 +16912,6 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-      <c r="H5">
-        <v>7</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>5</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>6</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <v>7</v>
-      </c>
-      <c r="L6">
-        <v>9</v>
-      </c>
-      <c r="M6">
         <v>1</v>
       </c>
     </row>
@@ -17121,47 +16985,68 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
         <v>1</v>
       </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3">
         <v>1</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -17173,25 +17058,34 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -17202,37 +17096,37 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6">
         <v>3</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J6">
+        <v>9</v>
+      </c>
+      <c r="K6">
         <v>7</v>
       </c>
-      <c r="K6">
-        <v>2</v>
-      </c>
       <c r="L6">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -17244,6 +17138,193 @@
 </file>
 
 <file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17402,7 +17483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17503,7 +17584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17620,7 +17701,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17676,117 +17757,6 @@
       </c>
       <c r="D4">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -18011,6 +17981,117 @@
 
 <file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -18103,7 +18184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18166,7 +18247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18249,7 +18330,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18345,7 +18426,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18448,7 +18529,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet86.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18534,7 +18615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet86.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet87.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18592,7 +18673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet87.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet88.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18723,7 +18804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet88.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet89.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18791,62 +18872,6 @@
         <v>1</v>
       </c>
       <c r="E4">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet89.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -19076,7 +19101,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="C1" s="1">
         <v>2023</v>
@@ -19084,9 +19109,9 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="B2">
         <v>1</v>
       </c>
     </row>
@@ -19095,6 +19120,9 @@
         <v>5</v>
       </c>
       <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
         <v>1</v>
       </c>
     </row>
@@ -19103,7 +19131,7 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -19115,6 +19143,59 @@
 </file>
 
 <file path=xl/worksheets/sheet91.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet92.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19175,7 +19256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet92.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet93.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19213,7 +19294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet93.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet94.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19271,7 +19352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet94.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet95.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19316,69 +19397,6 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet95.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
         <v>1</v>
       </c>
     </row>

</xml_diff>